<commit_message>
Update billing layout and responsive styles
</commit_message>
<xml_diff>
--- a/Billing Format.xlsx
+++ b/Billing Format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kotha Vitesh\Desktop\JewelDesk-master\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kotha Vitesh\Desktop\JewelDesk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC43236-D5DF-4630-ADF9-F8D6565E3917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7651BFFD-406B-424D-B48C-194EB4791E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,6 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>GSTIN: 37BINPG4036L2ZX</t>
-  </si>
-  <si>
     <t>Andhra Pradesh - 533 001.</t>
   </si>
   <si>
@@ -115,9 +112,6 @@
   </si>
   <si>
     <t>TERMS AND CONDITIONS</t>
-  </si>
-  <si>
-    <t>Call: 99082 66688</t>
   </si>
   <si>
     <t>Cash:</t>
@@ -136,15 +130,22 @@
 • All disputes are subject to Kakinada jurisdiction only
 • 100% Quality Guarantee but not Breakage guarantee</t>
   </si>
+  <si>
+    <t xml:space="preserve">GSTIN: </t>
+  </si>
+  <si>
+    <t>Phone No : 99082 66688</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -429,7 +430,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -472,25 +473,7 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -511,9 +494,6 @@
     <xf numFmtId="41" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -541,6 +521,105 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
@@ -628,95 +707,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -808,7 +824,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>420933</xdr:colOff>
+      <xdr:colOff>142311</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>143774</xdr:rowOff>
     </xdr:to>
@@ -1202,545 +1218,545 @@
   <sheetFormatPr defaultColWidth="9.296875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="5.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.09765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.3984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.69921875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.3984375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.69921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.19921875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.69921875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.69921875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.19921875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.796875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="11.69921875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5" style="1" customWidth="1"/>
     <col min="10" max="10" width="14.8984375" style="1" customWidth="1"/>
     <col min="11" max="16384" width="9.296875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44"/>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="77" t="s">
+      <c r="A1" s="70"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="92" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="93"/>
+    </row>
+    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="73"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="65"/>
+    </row>
+    <row r="3" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="73"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="78"/>
-    </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="47"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="39"/>
-    </row>
-    <row r="3" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="39"/>
+      <c r="J3" s="65"/>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="J4" s="39"/>
+      <c r="A4" s="73"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="99"/>
+      <c r="J4" s="100"/>
     </row>
     <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="50"/>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="41"/>
+      <c r="A5" s="76"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="78"/>
+      <c r="I5" s="66" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="67"/>
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="90"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="91"/>
+      <c r="I6" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="45"/>
+    </row>
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="14"/>
+    </row>
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="64"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
-      <c r="G6" s="64"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="20"/>
-    </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="66" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="67"/>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="18"/>
-    </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="67"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
-      <c r="H8" s="68"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
       <c r="I8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="J8" s="4"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="69" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
-      <c r="F9" s="70"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="71"/>
+      <c r="A9" s="36" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="38"/>
       <c r="I9" s="5"/>
       <c r="J9" s="6"/>
       <c r="N9"/>
     </row>
     <row r="10" spans="1:15" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="30" t="s">
+      <c r="A10" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="D10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="E10" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="F10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="G10" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="I10" s="22" t="s">
+      <c r="J10" s="24" t="s">
         <v>19</v>
-      </c>
-      <c r="J10" s="31" t="s">
-        <v>20</v>
       </c>
       <c r="O10"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="97"/>
+      <c r="E11" s="97"/>
+      <c r="F11" s="97"/>
+      <c r="G11" s="97"/>
       <c r="H11" s="12"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="16"/>
+      <c r="I11" s="94"/>
+      <c r="J11" s="30"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="98"/>
+      <c r="E12" s="98"/>
+      <c r="F12" s="98"/>
+      <c r="G12" s="98"/>
       <c r="H12" s="13"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="17"/>
+      <c r="I12" s="95"/>
+      <c r="J12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="98"/>
+      <c r="E13" s="98"/>
+      <c r="F13" s="98"/>
+      <c r="G13" s="98"/>
       <c r="H13" s="13"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="17"/>
+      <c r="I13" s="95"/>
+      <c r="J13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
       <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="98"/>
+      <c r="E14" s="98"/>
+      <c r="F14" s="98"/>
+      <c r="G14" s="98"/>
       <c r="H14" s="13"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="17"/>
+      <c r="I14" s="95"/>
+      <c r="J14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="98"/>
+      <c r="E15" s="98"/>
+      <c r="F15" s="98"/>
+      <c r="G15" s="98"/>
       <c r="H15" s="13"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="17"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="98"/>
+      <c r="F16" s="98"/>
+      <c r="G16" s="98"/>
       <c r="H16" s="13"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="17"/>
+      <c r="I16" s="95"/>
+      <c r="J16" s="31"/>
     </row>
     <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="98"/>
       <c r="H17" s="13"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="17"/>
+      <c r="I17" s="95"/>
+      <c r="J17" s="31"/>
     </row>
     <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="98"/>
+      <c r="E18" s="98"/>
+      <c r="F18" s="98"/>
+      <c r="G18" s="98"/>
       <c r="H18" s="13"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="17"/>
+      <c r="I18" s="95"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="19" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
       <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="98"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="98"/>
+      <c r="G19" s="98"/>
       <c r="H19" s="13"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="17"/>
+      <c r="I19" s="95"/>
+      <c r="J19" s="31"/>
     </row>
     <row r="20" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8"/>
       <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="98"/>
       <c r="H20" s="13"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="17"/>
+      <c r="I20" s="95"/>
+      <c r="J20" s="31"/>
     </row>
     <row r="21" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="98"/>
+      <c r="E21" s="98"/>
+      <c r="F21" s="98"/>
+      <c r="G21" s="98"/>
       <c r="H21" s="13"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="17"/>
+      <c r="I21" s="95"/>
+      <c r="J21" s="31"/>
     </row>
     <row r="22" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
       <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+      <c r="C22" s="96"/>
+      <c r="D22" s="98"/>
+      <c r="E22" s="98"/>
+      <c r="F22" s="98"/>
+      <c r="G22" s="98"/>
       <c r="H22" s="13"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="17"/>
+      <c r="I22" s="95"/>
+      <c r="J22" s="31"/>
     </row>
     <row r="23" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="98"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="98"/>
+      <c r="G23" s="98"/>
       <c r="H23" s="13"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="17"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="31"/>
     </row>
     <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="98"/>
+      <c r="E24" s="98"/>
+      <c r="F24" s="98"/>
+      <c r="G24" s="98"/>
       <c r="H24" s="13"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="17"/>
+      <c r="I24" s="95"/>
+      <c r="J24" s="31"/>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
       <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="98"/>
+      <c r="E25" s="98"/>
+      <c r="F25" s="98"/>
+      <c r="G25" s="98"/>
       <c r="H25" s="13"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="17"/>
+      <c r="I25" s="95"/>
+      <c r="J25" s="31"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="72" t="s">
+      <c r="A26" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="40"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="32"/>
+    </row>
+    <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="43"/>
+      <c r="J27" s="21"/>
+    </row>
+    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="83" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="84"/>
+      <c r="C28" s="84"/>
+      <c r="D28" s="84"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="84"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="84"/>
+      <c r="I28" s="85"/>
+      <c r="J28" s="21"/>
+    </row>
+    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="83" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="84"/>
+      <c r="C29" s="84"/>
+      <c r="D29" s="84"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="84"/>
+      <c r="G29" s="84"/>
+      <c r="H29" s="84"/>
+      <c r="I29" s="85"/>
+      <c r="J29" s="21"/>
+    </row>
+    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="83" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="84"/>
+      <c r="C30" s="84"/>
+      <c r="D30" s="84"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="84"/>
+      <c r="G30" s="84"/>
+      <c r="H30" s="84"/>
+      <c r="I30" s="85"/>
+      <c r="J30" s="21"/>
+    </row>
+    <row r="31" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="73"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="27"/>
-    </row>
-    <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="74" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="75"/>
-      <c r="C27" s="75"/>
-      <c r="D27" s="75"/>
-      <c r="E27" s="75"/>
-      <c r="F27" s="75"/>
-      <c r="G27" s="75"/>
-      <c r="H27" s="75"/>
-      <c r="I27" s="76"/>
-      <c r="J27" s="28"/>
-    </row>
-    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="57" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28" s="58"/>
-      <c r="C28" s="58"/>
-      <c r="D28" s="58"/>
-      <c r="E28" s="58"/>
-      <c r="F28" s="58"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="58"/>
-      <c r="I28" s="59"/>
-      <c r="J28" s="28"/>
-    </row>
-    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="58"/>
-      <c r="C29" s="58"/>
-      <c r="D29" s="58"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="58"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="58"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="28"/>
-    </row>
-    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" s="58"/>
-      <c r="C30" s="58"/>
-      <c r="D30" s="58"/>
-      <c r="E30" s="58"/>
-      <c r="F30" s="58"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="58"/>
-      <c r="I30" s="59"/>
-      <c r="J30" s="28"/>
-    </row>
-    <row r="31" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="60" t="s">
-        <v>22</v>
-      </c>
-      <c r="B31" s="61"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
-      <c r="F31" s="61"/>
-      <c r="G31" s="61"/>
-      <c r="H31" s="61"/>
-      <c r="I31" s="62"/>
-      <c r="J31" s="29"/>
+      <c r="B31" s="87"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="87"/>
+      <c r="F31" s="87"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="87"/>
+      <c r="I31" s="88"/>
+      <c r="J31" s="22"/>
     </row>
     <row r="32" spans="1:10" ht="22" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="53" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="54"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="55"/>
-      <c r="H32" s="55"/>
-      <c r="I32" s="55"/>
-      <c r="J32" s="56"/>
+      <c r="A32" s="79" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" s="80"/>
+      <c r="C32" s="81"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="81"/>
+      <c r="J32" s="82"/>
     </row>
     <row r="33" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="32"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="82" t="s">
+      <c r="A33" s="25"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="49" t="s">
+        <v>3</v>
+      </c>
+      <c r="G33" s="50"/>
+      <c r="H33" s="50"/>
+      <c r="I33" s="50"/>
+      <c r="J33" s="51"/>
+    </row>
+    <row r="34" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="28"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="G33" s="83"/>
-      <c r="H33" s="83"/>
-      <c r="I33" s="83"/>
-      <c r="J33" s="84"/>
-    </row>
-    <row r="34" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="35"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="85" t="s">
+      <c r="G34" s="53"/>
+      <c r="H34" s="53"/>
+      <c r="I34" s="53"/>
+      <c r="J34" s="54"/>
+    </row>
+    <row r="35" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="28"/>
+      <c r="B35" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
+      <c r="J35" s="54"/>
+    </row>
+    <row r="36" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="28"/>
+      <c r="B36" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="57"/>
+    </row>
+    <row r="37" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="28"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="57"/>
+    </row>
+    <row r="38" spans="1:12" ht="21.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="46"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="86"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="86"/>
-      <c r="J34" s="87"/>
-    </row>
-    <row r="35" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="35"/>
-      <c r="B35" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="94"/>
-      <c r="D35" s="94"/>
-      <c r="E35" s="95"/>
-      <c r="F35" s="85"/>
-      <c r="G35" s="86"/>
-      <c r="H35" s="86"/>
-      <c r="I35" s="86"/>
-      <c r="J35" s="87"/>
-    </row>
-    <row r="36" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="35"/>
-      <c r="B36" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36" s="94"/>
-      <c r="D36" s="94"/>
-      <c r="E36" s="95"/>
-      <c r="F36" s="88"/>
-      <c r="G36" s="89"/>
-      <c r="H36" s="89"/>
-      <c r="I36" s="89"/>
-      <c r="J36" s="90"/>
-    </row>
-    <row r="37" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="35"/>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="88"/>
-      <c r="G37" s="89"/>
-      <c r="H37" s="89"/>
-      <c r="I37" s="89"/>
-      <c r="J37" s="90"/>
-    </row>
-    <row r="38" spans="1:12" ht="21.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="79"/>
-      <c r="B38" s="80"/>
-      <c r="C38" s="80"/>
-      <c r="D38" s="80"/>
-      <c r="E38" s="81"/>
-      <c r="F38" s="91" t="s">
-        <v>6</v>
-      </c>
-      <c r="G38" s="92"/>
-      <c r="H38" s="92"/>
-      <c r="I38" s="92"/>
-      <c r="J38" s="93"/>
+      <c r="G38" s="59"/>
+      <c r="H38" s="59"/>
+      <c r="I38" s="59"/>
+      <c r="J38" s="60"/>
     </row>
     <row r="41" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="42"/>
+      <c r="B41" s="68"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -1752,7 +1768,7 @@
     </row>
     <row r="42" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
-      <c r="B42" s="42"/>
+      <c r="B42" s="68"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -1764,7 +1780,7 @@
     </row>
     <row r="43" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
-      <c r="B43" s="42"/>
+      <c r="B43" s="68"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -1776,15 +1792,15 @@
     </row>
     <row r="44" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
-      <c r="B44" s="42"/>
-      <c r="C44" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="D44" s="43"/>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="43"/>
+      <c r="B44" s="68"/>
+      <c r="C44" s="69" t="s">
+        <v>29</v>
+      </c>
+      <c r="D44" s="69"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="69"/>
+      <c r="G44" s="69"/>
+      <c r="H44" s="69"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44"/>
@@ -1792,7 +1808,7 @@
     </row>
     <row r="45" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
-      <c r="B45" s="42"/>
+      <c r="B45" s="68"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -1804,270 +1820,270 @@
     </row>
     <row r="46" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
-      <c r="B46" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="37"/>
-      <c r="I46" s="37"/>
-      <c r="J46" s="37"/>
+      <c r="B46" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="63"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="63"/>
+      <c r="F46" s="63"/>
+      <c r="G46" s="63"/>
+      <c r="H46" s="63"/>
+      <c r="I46" s="63"/>
+      <c r="J46" s="63"/>
     </row>
     <row r="47" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
-      <c r="B47" s="37"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="37"/>
-      <c r="J47" s="37"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="63"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="63"/>
+      <c r="G47" s="63"/>
+      <c r="H47" s="63"/>
+      <c r="I47" s="63"/>
+      <c r="J47" s="63"/>
     </row>
     <row r="48" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
-      <c r="B48" s="37"/>
-      <c r="C48" s="37"/>
-      <c r="D48" s="37"/>
-      <c r="E48" s="37"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="37"/>
-      <c r="I48" s="37"/>
-      <c r="J48" s="37"/>
+      <c r="B48" s="63"/>
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="63"/>
+      <c r="F48" s="63"/>
+      <c r="G48" s="63"/>
+      <c r="H48" s="63"/>
+      <c r="I48" s="63"/>
+      <c r="J48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
-      <c r="B49" s="37"/>
-      <c r="C49" s="37"/>
-      <c r="D49" s="37"/>
-      <c r="E49" s="37"/>
-      <c r="F49" s="37"/>
-      <c r="G49" s="37"/>
-      <c r="H49" s="37"/>
-      <c r="I49" s="37"/>
-      <c r="J49" s="37"/>
+      <c r="B49" s="63"/>
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
-      <c r="B50" s="37"/>
-      <c r="C50" s="37"/>
-      <c r="D50" s="37"/>
-      <c r="E50" s="37"/>
-      <c r="F50" s="37"/>
-      <c r="G50" s="37"/>
-      <c r="H50" s="37"/>
-      <c r="I50" s="37"/>
-      <c r="J50" s="37"/>
+      <c r="B50" s="63"/>
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="63"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="63"/>
+      <c r="H50" s="63"/>
+      <c r="I50" s="63"/>
+      <c r="J50" s="63"/>
     </row>
     <row r="51" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
-      <c r="B51" s="37"/>
-      <c r="C51" s="37"/>
-      <c r="D51" s="37"/>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="37"/>
-      <c r="I51" s="37"/>
-      <c r="J51" s="37"/>
+      <c r="B51" s="63"/>
+      <c r="C51" s="63"/>
+      <c r="D51" s="63"/>
+      <c r="E51" s="63"/>
+      <c r="F51" s="63"/>
+      <c r="G51" s="63"/>
+      <c r="H51" s="63"/>
+      <c r="I51" s="63"/>
+      <c r="J51" s="63"/>
       <c r="K51"/>
     </row>
     <row r="52" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
-      <c r="B52" s="37"/>
-      <c r="C52" s="37"/>
-      <c r="D52" s="37"/>
-      <c r="E52" s="37"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="37"/>
-      <c r="I52" s="37"/>
-      <c r="J52" s="37"/>
+      <c r="B52" s="63"/>
+      <c r="C52" s="63"/>
+      <c r="D52" s="63"/>
+      <c r="E52" s="63"/>
+      <c r="F52" s="63"/>
+      <c r="G52" s="63"/>
+      <c r="H52" s="63"/>
+      <c r="I52" s="63"/>
+      <c r="J52" s="63"/>
     </row>
     <row r="53" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-      <c r="E53" s="37"/>
-      <c r="F53" s="37"/>
-      <c r="G53" s="37"/>
-      <c r="H53" s="37"/>
-      <c r="I53" s="37"/>
-      <c r="J53" s="37"/>
+      <c r="B53" s="63"/>
+      <c r="C53" s="63"/>
+      <c r="D53" s="63"/>
+      <c r="E53" s="63"/>
+      <c r="F53" s="63"/>
+      <c r="G53" s="63"/>
+      <c r="H53" s="63"/>
+      <c r="I53" s="63"/>
+      <c r="J53" s="63"/>
     </row>
     <row r="54" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
-      <c r="B54" s="37"/>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="37"/>
-      <c r="F54" s="37"/>
-      <c r="G54" s="37"/>
-      <c r="H54" s="37"/>
-      <c r="I54" s="37"/>
-      <c r="J54" s="37"/>
+      <c r="B54" s="63"/>
+      <c r="C54" s="63"/>
+      <c r="D54" s="63"/>
+      <c r="E54" s="63"/>
+      <c r="F54" s="63"/>
+      <c r="G54" s="63"/>
+      <c r="H54" s="63"/>
+      <c r="I54" s="63"/>
+      <c r="J54" s="63"/>
     </row>
     <row r="55" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
-      <c r="B55" s="37"/>
-      <c r="C55" s="37"/>
-      <c r="D55" s="37"/>
-      <c r="E55" s="37"/>
-      <c r="F55" s="37"/>
-      <c r="G55" s="37"/>
-      <c r="H55" s="37"/>
-      <c r="I55" s="37"/>
-      <c r="J55" s="37"/>
+      <c r="B55" s="63"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="63"/>
+      <c r="E55" s="63"/>
+      <c r="F55" s="63"/>
+      <c r="G55" s="63"/>
+      <c r="H55" s="63"/>
+      <c r="I55" s="63"/>
+      <c r="J55" s="63"/>
     </row>
     <row r="56" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
-      <c r="B56" s="37"/>
-      <c r="C56" s="37"/>
-      <c r="D56" s="37"/>
-      <c r="E56" s="37"/>
-      <c r="F56" s="37"/>
-      <c r="G56" s="37"/>
-      <c r="H56" s="37"/>
-      <c r="I56" s="37"/>
-      <c r="J56" s="37"/>
+      <c r="B56" s="63"/>
+      <c r="C56" s="63"/>
+      <c r="D56" s="63"/>
+      <c r="E56" s="63"/>
+      <c r="F56" s="63"/>
+      <c r="G56" s="63"/>
+      <c r="H56" s="63"/>
+      <c r="I56" s="63"/>
+      <c r="J56" s="63"/>
     </row>
     <row r="57" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
-      <c r="B57" s="37"/>
-      <c r="C57" s="37"/>
-      <c r="D57" s="37"/>
-      <c r="E57" s="37"/>
-      <c r="F57" s="37"/>
-      <c r="G57" s="37"/>
-      <c r="H57" s="37"/>
-      <c r="I57" s="37"/>
-      <c r="J57" s="37"/>
+      <c r="B57" s="63"/>
+      <c r="C57" s="63"/>
+      <c r="D57" s="63"/>
+      <c r="E57" s="63"/>
+      <c r="F57" s="63"/>
+      <c r="G57" s="63"/>
+      <c r="H57" s="63"/>
+      <c r="I57" s="63"/>
+      <c r="J57" s="63"/>
     </row>
     <row r="58" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
-      <c r="B58" s="37"/>
-      <c r="C58" s="37"/>
-      <c r="D58" s="37"/>
-      <c r="E58" s="37"/>
-      <c r="F58" s="37"/>
-      <c r="G58" s="37"/>
-      <c r="H58" s="37"/>
-      <c r="I58" s="37"/>
-      <c r="J58" s="37"/>
+      <c r="B58" s="63"/>
+      <c r="C58" s="63"/>
+      <c r="D58" s="63"/>
+      <c r="E58" s="63"/>
+      <c r="F58" s="63"/>
+      <c r="G58" s="63"/>
+      <c r="H58" s="63"/>
+      <c r="I58" s="63"/>
+      <c r="J58" s="63"/>
     </row>
     <row r="59" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
-      <c r="B59" s="37"/>
-      <c r="C59" s="37"/>
-      <c r="D59" s="37"/>
-      <c r="E59" s="37"/>
-      <c r="F59" s="37"/>
-      <c r="G59" s="37"/>
-      <c r="H59" s="37"/>
-      <c r="I59" s="37"/>
-      <c r="J59" s="37"/>
+      <c r="B59" s="63"/>
+      <c r="C59" s="63"/>
+      <c r="D59" s="63"/>
+      <c r="E59" s="63"/>
+      <c r="F59" s="63"/>
+      <c r="G59" s="63"/>
+      <c r="H59" s="63"/>
+      <c r="I59" s="63"/>
+      <c r="J59" s="63"/>
     </row>
     <row r="60" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
-      <c r="B60" s="37"/>
-      <c r="C60" s="37"/>
-      <c r="D60" s="37"/>
-      <c r="E60" s="37"/>
-      <c r="F60" s="37"/>
-      <c r="G60" s="37"/>
-      <c r="H60" s="37"/>
-      <c r="I60" s="37"/>
-      <c r="J60" s="37"/>
+      <c r="B60" s="63"/>
+      <c r="C60" s="63"/>
+      <c r="D60" s="63"/>
+      <c r="E60" s="63"/>
+      <c r="F60" s="63"/>
+      <c r="G60" s="63"/>
+      <c r="H60" s="63"/>
+      <c r="I60" s="63"/>
+      <c r="J60" s="63"/>
     </row>
     <row r="61" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
-      <c r="B61" s="37"/>
-      <c r="C61" s="37"/>
-      <c r="D61" s="37"/>
-      <c r="E61" s="37"/>
-      <c r="F61" s="37"/>
-      <c r="G61" s="37"/>
-      <c r="H61" s="37"/>
-      <c r="I61" s="37"/>
-      <c r="J61" s="37"/>
+      <c r="B61" s="63"/>
+      <c r="C61" s="63"/>
+      <c r="D61" s="63"/>
+      <c r="E61" s="63"/>
+      <c r="F61" s="63"/>
+      <c r="G61" s="63"/>
+      <c r="H61" s="63"/>
+      <c r="I61" s="63"/>
+      <c r="J61" s="63"/>
     </row>
     <row r="62" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
-      <c r="B62" s="37"/>
-      <c r="C62" s="37"/>
-      <c r="D62" s="37"/>
-      <c r="E62" s="37"/>
-      <c r="F62" s="37"/>
-      <c r="G62" s="37"/>
-      <c r="H62" s="37"/>
-      <c r="I62" s="37"/>
-      <c r="J62" s="37"/>
+      <c r="B62" s="63"/>
+      <c r="C62" s="63"/>
+      <c r="D62" s="63"/>
+      <c r="E62" s="63"/>
+      <c r="F62" s="63"/>
+      <c r="G62" s="63"/>
+      <c r="H62" s="63"/>
+      <c r="I62" s="63"/>
+      <c r="J62" s="63"/>
     </row>
     <row r="63" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
-      <c r="B63" s="37"/>
-      <c r="C63" s="37"/>
-      <c r="D63" s="37"/>
-      <c r="E63" s="37"/>
-      <c r="F63" s="37"/>
-      <c r="G63" s="37"/>
-      <c r="H63" s="37"/>
-      <c r="I63" s="37"/>
-      <c r="J63" s="37"/>
+      <c r="B63" s="63"/>
+      <c r="C63" s="63"/>
+      <c r="D63" s="63"/>
+      <c r="E63" s="63"/>
+      <c r="F63" s="63"/>
+      <c r="G63" s="63"/>
+      <c r="H63" s="63"/>
+      <c r="I63" s="63"/>
+      <c r="J63" s="63"/>
     </row>
     <row r="64" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
-      <c r="B64" s="37"/>
-      <c r="C64" s="37"/>
-      <c r="D64" s="37"/>
-      <c r="E64" s="37"/>
-      <c r="F64" s="37"/>
-      <c r="G64" s="37"/>
-      <c r="H64" s="37"/>
-      <c r="I64" s="37"/>
-      <c r="J64" s="37"/>
+      <c r="B64" s="63"/>
+      <c r="C64" s="63"/>
+      <c r="D64" s="63"/>
+      <c r="E64" s="63"/>
+      <c r="F64" s="63"/>
+      <c r="G64" s="63"/>
+      <c r="H64" s="63"/>
+      <c r="I64" s="63"/>
+      <c r="J64" s="63"/>
     </row>
     <row r="65" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
-      <c r="B65" s="37"/>
-      <c r="C65" s="37"/>
-      <c r="D65" s="37"/>
-      <c r="E65" s="37"/>
-      <c r="F65" s="37"/>
-      <c r="G65" s="37"/>
-      <c r="H65" s="37"/>
-      <c r="I65" s="37"/>
-      <c r="J65" s="37"/>
+      <c r="B65" s="63"/>
+      <c r="C65" s="63"/>
+      <c r="D65" s="63"/>
+      <c r="E65" s="63"/>
+      <c r="F65" s="63"/>
+      <c r="G65" s="63"/>
+      <c r="H65" s="63"/>
+      <c r="I65" s="63"/>
+      <c r="J65" s="63"/>
     </row>
     <row r="66" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
-      <c r="B66" s="37"/>
-      <c r="C66" s="37"/>
-      <c r="D66" s="37"/>
-      <c r="E66" s="37"/>
-      <c r="F66" s="37"/>
-      <c r="G66" s="37"/>
-      <c r="H66" s="37"/>
-      <c r="I66" s="37"/>
-      <c r="J66" s="37"/>
+      <c r="B66" s="63"/>
+      <c r="C66" s="63"/>
+      <c r="D66" s="63"/>
+      <c r="E66" s="63"/>
+      <c r="F66" s="63"/>
+      <c r="G66" s="63"/>
+      <c r="H66" s="63"/>
+      <c r="I66" s="63"/>
+      <c r="J66" s="63"/>
     </row>
     <row r="67" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
-      <c r="B67" s="37"/>
-      <c r="C67" s="37"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="37"/>
-      <c r="F67" s="37"/>
-      <c r="G67" s="37"/>
-      <c r="H67" s="37"/>
-      <c r="I67" s="37"/>
-      <c r="J67" s="37"/>
+      <c r="B67" s="63"/>
+      <c r="C67" s="63"/>
+      <c r="D67" s="63"/>
+      <c r="E67" s="63"/>
+      <c r="F67" s="63"/>
+      <c r="G67" s="63"/>
+      <c r="H67" s="63"/>
+      <c r="I67" s="63"/>
+      <c r="J67" s="63"/>
     </row>
     <row r="68" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
@@ -2155,24 +2171,10 @@
       <c r="M74"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="F33:J33"/>
-    <mergeCell ref="F34:J34"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="F36:J36"/>
-    <mergeCell ref="F37:J37"/>
-    <mergeCell ref="F38:J38"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:I27"/>
-    <mergeCell ref="I1:J1"/>
+  <mergeCells count="31">
+    <mergeCell ref="B46:J67"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="B46:J67"/>
     <mergeCell ref="I3:J3"/>
-    <mergeCell ref="I4:J4"/>
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="C44:H44"/>
@@ -2185,11 +2187,26 @@
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A7:H7"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="F33:J33"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="F36:J36"/>
+    <mergeCell ref="F37:J37"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="I4:J4"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="94" fitToHeight="2" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>